<commit_message>
Workbook: add per-month MARKETING/ANZIL and GoLuna-fixed subtotal rows
Cost Forecast sheet now shows the split explicitly above the monthly total:
- MARKETING / ANZIL monthly total (setup + retainer + media + mgmt):
  3,240 / 18,870 / 30,370 / 34,970 / 0... = 87,450
- GoLuna fixed monthly total: 24,427 / 9,314... = 159,281
- Monthly total redefined as fixed + marketing (values unchanged)

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
+++ b/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="93">
   <si>
     <t xml:space="preserve">GoLuna — Path C (Anzil) Month-by-Month Cost Forecast (USD)</t>
   </si>
@@ -140,7 +140,13 @@
     <t xml:space="preserve">Anzil management (15% of media)</t>
   </si>
   <si>
-    <t xml:space="preserve">Monthly total</t>
+    <t xml:space="preserve">MARKETING / ANZIL — monthly total (setup + retainer + media + mgmt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GoLuna fixed — monthly total (salaries, platform, security, one-times)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly total (fixed + marketing)</t>
   </si>
   <si>
     <t xml:space="preserve">Cumulative</t>
@@ -447,7 +453,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -501,6 +507,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -796,7 +806,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1712,185 +1722,281 @@
         <v>39</v>
       </c>
       <c r="B29" s="14" t="n">
-        <f aca="false">SUM(B12:B28)</f>
-        <v>27667</v>
+        <f aca="false">SUM(B25:B28)</f>
+        <v>3240</v>
       </c>
       <c r="C29" s="14" t="n">
-        <f aca="false">SUM(C12:C28)</f>
-        <v>28184</v>
+        <f aca="false">SUM(C25:C28)</f>
+        <v>18870</v>
       </c>
       <c r="D29" s="14" t="n">
-        <f aca="false">SUM(D12:D28)</f>
-        <v>39684</v>
+        <f aca="false">SUM(D25:D28)</f>
+        <v>30370</v>
       </c>
       <c r="E29" s="14" t="n">
-        <f aca="false">SUM(E12:E28)</f>
-        <v>44284</v>
+        <f aca="false">SUM(E25:E28)</f>
+        <v>34970</v>
       </c>
       <c r="F29" s="14" t="n">
-        <f aca="false">SUM(F12:F28)</f>
-        <v>9314</v>
+        <f aca="false">SUM(F25:F28)</f>
+        <v>0</v>
       </c>
       <c r="G29" s="14" t="n">
-        <f aca="false">SUM(G12:G28)</f>
-        <v>9314</v>
+        <f aca="false">SUM(G25:G28)</f>
+        <v>0</v>
       </c>
       <c r="H29" s="14" t="n">
-        <f aca="false">SUM(H12:H28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(H25:H28)</f>
+        <v>0</v>
       </c>
       <c r="I29" s="14" t="n">
-        <f aca="false">SUM(I12:I28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(I25:I28)</f>
+        <v>0</v>
       </c>
       <c r="J29" s="14" t="n">
-        <f aca="false">SUM(J12:J28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(J25:J28)</f>
+        <v>0</v>
       </c>
       <c r="K29" s="14" t="n">
-        <f aca="false">SUM(K12:K28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(K25:K28)</f>
+        <v>0</v>
       </c>
       <c r="L29" s="14" t="n">
-        <f aca="false">SUM(L12:L28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(L25:L28)</f>
+        <v>0</v>
       </c>
       <c r="M29" s="14" t="n">
-        <f aca="false">SUM(M12:M28)</f>
-        <v>14714</v>
+        <f aca="false">SUM(M25:M28)</f>
+        <v>0</v>
       </c>
       <c r="N29" s="14" t="n">
-        <f aca="false">SUM(N12:N28)</f>
-        <v>246731</v>
+        <f aca="false">SUM(N25:N28)</f>
+        <v>87450</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B30" s="6" t="n">
-        <f aca="false">B29</f>
-        <v>27667</v>
-      </c>
-      <c r="C30" s="6" t="n">
-        <f aca="false">B30+C29</f>
-        <v>55851</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <f aca="false">C30+D29</f>
-        <v>95535</v>
-      </c>
-      <c r="E30" s="6" t="n">
-        <f aca="false">D30+E29</f>
-        <v>139819</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <f aca="false">E30+F29</f>
-        <v>149133</v>
-      </c>
-      <c r="G30" s="6" t="n">
-        <f aca="false">F30+G29</f>
-        <v>158447</v>
-      </c>
-      <c r="H30" s="6" t="n">
-        <f aca="false">G30+H29</f>
-        <v>173161</v>
-      </c>
-      <c r="I30" s="6" t="n">
-        <f aca="false">H30+I29</f>
-        <v>187875</v>
-      </c>
-      <c r="J30" s="6" t="n">
-        <f aca="false">I30+J29</f>
-        <v>202589</v>
-      </c>
-      <c r="K30" s="6" t="n">
-        <f aca="false">J30+K29</f>
-        <v>217303</v>
-      </c>
-      <c r="L30" s="6" t="n">
-        <f aca="false">K30+L29</f>
-        <v>232017</v>
-      </c>
-      <c r="M30" s="6" t="n">
-        <f aca="false">L30+M29</f>
-        <v>246731</v>
+      <c r="B30" s="15" t="n">
+        <f aca="false">SUM(B12:B24)</f>
+        <v>24427</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <f aca="false">SUM(C12:C24)</f>
+        <v>9314</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <f aca="false">SUM(D12:D24)</f>
+        <v>9314</v>
+      </c>
+      <c r="E30" s="15" t="n">
+        <f aca="false">SUM(E12:E24)</f>
+        <v>9314</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <f aca="false">SUM(F12:F24)</f>
+        <v>9314</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <f aca="false">SUM(G12:G24)</f>
+        <v>9314</v>
+      </c>
+      <c r="H30" s="15" t="n">
+        <f aca="false">SUM(H12:H24)</f>
+        <v>14714</v>
+      </c>
+      <c r="I30" s="15" t="n">
+        <f aca="false">SUM(I12:I24)</f>
+        <v>14714</v>
+      </c>
+      <c r="J30" s="15" t="n">
+        <f aca="false">SUM(J12:J24)</f>
+        <v>14714</v>
+      </c>
+      <c r="K30" s="15" t="n">
+        <f aca="false">SUM(K12:K24)</f>
+        <v>14714</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <f aca="false">SUM(L12:L24)</f>
+        <v>14714</v>
+      </c>
+      <c r="M30" s="15" t="n">
+        <f aca="false">SUM(M12:M24)</f>
+        <v>14714</v>
+      </c>
+      <c r="N30" s="15" t="n">
+        <f aca="false">SUM(N12:N24)</f>
+        <v>159281</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B31" s="6" t="n">
-        <f aca="false">$B$6-B30</f>
+      <c r="B31" s="15" t="n">
+        <f aca="false">B29+B30</f>
+        <v>27667</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <f aca="false">C29+C30</f>
+        <v>28184</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <f aca="false">D29+D30</f>
+        <v>39684</v>
+      </c>
+      <c r="E31" s="15" t="n">
+        <f aca="false">E29+E30</f>
+        <v>44284</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <f aca="false">F29+F30</f>
+        <v>9314</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <f aca="false">G29+G30</f>
+        <v>9314</v>
+      </c>
+      <c r="H31" s="15" t="n">
+        <f aca="false">H29+H30</f>
+        <v>14714</v>
+      </c>
+      <c r="I31" s="15" t="n">
+        <f aca="false">I29+I30</f>
+        <v>14714</v>
+      </c>
+      <c r="J31" s="15" t="n">
+        <f aca="false">J29+J30</f>
+        <v>14714</v>
+      </c>
+      <c r="K31" s="15" t="n">
+        <f aca="false">K29+K30</f>
+        <v>14714</v>
+      </c>
+      <c r="L31" s="15" t="n">
+        <f aca="false">L29+L30</f>
+        <v>14714</v>
+      </c>
+      <c r="M31" s="15" t="n">
+        <f aca="false">M29+M30</f>
+        <v>14714</v>
+      </c>
+      <c r="N31" s="15" t="n">
+        <f aca="false">N29+N30</f>
+        <v>246731</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="6" t="n">
+        <f aca="false">B31</f>
+        <v>27667</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <f aca="false">B32+C31</f>
+        <v>55851</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <f aca="false">C32+D31</f>
+        <v>95535</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <f aca="false">D32+E31</f>
+        <v>139819</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <f aca="false">E32+F31</f>
+        <v>149133</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <f aca="false">F32+G31</f>
+        <v>158447</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <f aca="false">G32+H31</f>
+        <v>173161</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <f aca="false">H32+I31</f>
+        <v>187875</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <f aca="false">I32+J31</f>
+        <v>202589</v>
+      </c>
+      <c r="K32" s="6" t="n">
+        <f aca="false">J32+K31</f>
+        <v>217303</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <f aca="false">K32+L31</f>
+        <v>232017</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <f aca="false">L32+M31</f>
+        <v>246731</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <f aca="false">$B$6-B32</f>
         <v>210428.238095238</v>
       </c>
-      <c r="C31" s="6" t="n">
-        <f aca="false">$B$6-C30</f>
+      <c r="C33" s="6" t="n">
+        <f aca="false">$B$6-C32</f>
         <v>182244.238095238</v>
       </c>
-      <c r="D31" s="6" t="n">
-        <f aca="false">$B$6-D30</f>
+      <c r="D33" s="6" t="n">
+        <f aca="false">$B$6-D32</f>
         <v>142560.238095238</v>
       </c>
-      <c r="E31" s="6" t="n">
-        <f aca="false">$B$6-E30</f>
+      <c r="E33" s="6" t="n">
+        <f aca="false">$B$6-E32</f>
         <v>98276.2380952381</v>
       </c>
-      <c r="F31" s="6" t="n">
-        <f aca="false">$B$6-F30</f>
+      <c r="F33" s="6" t="n">
+        <f aca="false">$B$6-F32</f>
         <v>88962.2380952381</v>
       </c>
-      <c r="G31" s="6" t="n">
-        <f aca="false">$B$6-G30</f>
+      <c r="G33" s="6" t="n">
+        <f aca="false">$B$6-G32</f>
         <v>79648.2380952381</v>
       </c>
-      <c r="H31" s="6" t="n">
-        <f aca="false">$B$6-H30</f>
+      <c r="H33" s="6" t="n">
+        <f aca="false">$B$6-H32</f>
         <v>64934.2380952381</v>
       </c>
-      <c r="I31" s="6" t="n">
-        <f aca="false">$B$6-I30</f>
+      <c r="I33" s="6" t="n">
+        <f aca="false">$B$6-I32</f>
         <v>50220.2380952381</v>
       </c>
-      <c r="J31" s="6" t="n">
-        <f aca="false">$B$6-J30</f>
+      <c r="J33" s="6" t="n">
+        <f aca="false">$B$6-J32</f>
         <v>35506.2380952381</v>
       </c>
-      <c r="K31" s="6" t="n">
-        <f aca="false">$B$6-K30</f>
+      <c r="K33" s="6" t="n">
+        <f aca="false">$B$6-K32</f>
         <v>20792.2380952381</v>
       </c>
-      <c r="L31" s="6" t="n">
-        <f aca="false">$B$6-L30</f>
+      <c r="L33" s="6" t="n">
+        <f aca="false">$B$6-L32</f>
         <v>6078.23809523811</v>
       </c>
-      <c r="M31" s="6" t="n">
-        <f aca="false">$B$6-M30</f>
+      <c r="M33" s="6" t="n">
+        <f aca="false">$B$6-M32</f>
         <v>-8635.76190476189</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B35" s="6" t="n">
-        <f aca="false">N25+N26+N27+N28</f>
-        <v>87450</v>
-      </c>
-    </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="B36" s="6" t="n">
-        <f aca="false">B7</f>
-        <v>95238.0952380952</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,8 +2004,8 @@
         <v>45</v>
       </c>
       <c r="B37" s="6" t="n">
-        <f aca="false">B7-B35</f>
-        <v>7788.09523809524</v>
+        <f aca="false">N25+N26+N27+N28</f>
+        <v>87450</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1907,8 +2013,8 @@
         <v>46</v>
       </c>
       <c r="B38" s="6" t="n">
-        <f aca="false">B9</f>
-        <v>100000</v>
+        <f aca="false">B7</f>
+        <v>95238.0952380952</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1916,8 +2022,8 @@
         <v>47</v>
       </c>
       <c r="B39" s="6" t="n">
-        <f aca="false">B9-B35</f>
-        <v>12550</v>
+        <f aca="false">B7-B37</f>
+        <v>7788.09523809524</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,8 +2031,8 @@
         <v>48</v>
       </c>
       <c r="B40" s="6" t="n">
-        <f aca="false">B25+C26+C27+C28</f>
-        <v>22110</v>
+        <f aca="false">B9</f>
+        <v>100000</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1934,8 +2040,8 @@
         <v>49</v>
       </c>
       <c r="B41" s="6" t="n">
-        <f aca="false">B35-B40</f>
-        <v>65340</v>
+        <f aca="false">B9-B37</f>
+        <v>12550</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1943,7 +2049,25 @@
         <v>50</v>
       </c>
       <c r="B42" s="6" t="n">
-        <f aca="false">B40+D26+D27+D28</f>
+        <f aca="false">B25+C26+C27+C28</f>
+        <v>22110</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" s="6" t="n">
+        <f aca="false">B37-B42</f>
+        <v>65340</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="6" t="n">
+        <f aca="false">B42+D26+D27+D28</f>
         <v>52480</v>
       </c>
     </row>
@@ -1976,7 +2100,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1988,7 +2112,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2005,7 +2129,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>30</v>
@@ -2013,7 +2137,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>20</v>
@@ -2021,15 +2145,15 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <v>0.75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>0.515</v>
@@ -2037,7 +2161,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>0.28</v>
@@ -2045,7 +2169,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>0.39</v>
@@ -2053,28 +2177,28 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" s="16" t="n">
-        <f aca="false">'Cost Forecast'!H29</f>
+        <v>61</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <f aca="false">'Cost Forecast'!H31</f>
         <v>14714</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>13</v>
@@ -2083,156 +2207,156 @@
         <v>14</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="16" t="n">
+        <v>68</v>
+      </c>
+      <c r="B14" s="17" t="n">
         <f aca="false">'Cost Forecast'!B27</f>
         <v>0</v>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="17" t="n">
         <f aca="false">'Cost Forecast'!C27</f>
         <v>15000</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">'Cost Forecast'!D27</f>
         <v>25000</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="17" t="n">
         <f aca="false">'Cost Forecast'!E27</f>
         <v>29000</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="17" t="n">
         <f aca="false">'Cost Forecast'!F27</f>
         <v>0</v>
       </c>
-      <c r="G14" s="16" t="n">
+      <c r="G14" s="17" t="n">
         <f aca="false">'Cost Forecast'!G27</f>
         <v>0</v>
       </c>
-      <c r="H14" s="16" t="n">
+      <c r="H14" s="17" t="n">
         <f aca="false">'Cost Forecast'!H27</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="17" t="n">
+        <v>69</v>
+      </c>
+      <c r="B15" s="18" t="n">
         <f aca="false">B14/$B$6</f>
         <v>0</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <f aca="false">C14/$B$6</f>
         <v>750</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="18" t="n">
         <f aca="false">D14/$B$6</f>
         <v>1250</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="18" t="n">
         <f aca="false">E14/$B$6</f>
         <v>1450</v>
       </c>
-      <c r="F15" s="17" t="n">
+      <c r="F15" s="18" t="n">
         <f aca="false">F14/$B$6</f>
         <v>0</v>
       </c>
-      <c r="G15" s="17" t="n">
+      <c r="G15" s="18" t="n">
         <f aca="false">G14/$B$6</f>
         <v>0</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="H15" s="18" t="n">
         <f aca="false">H14/$B$6</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="B16" s="18" t="n">
         <f aca="false">B15</f>
         <v>0</v>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <f aca="false">B16+C15</f>
         <v>750</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <f aca="false">C16+D15</f>
         <v>2000</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="18" t="n">
         <f aca="false">D16+E15</f>
         <v>3450</v>
       </c>
-      <c r="F16" s="17" t="n">
+      <c r="F16" s="18" t="n">
         <f aca="false">E16+F15</f>
         <v>3450</v>
       </c>
-      <c r="G16" s="17" t="n">
+      <c r="G16" s="18" t="n">
         <f aca="false">F16+G15</f>
         <v>3450</v>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="H16" s="18" t="n">
         <f aca="false">G16+H15</f>
         <v>3450</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
+      <c r="A18" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="B19" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C19" s="18" t="n">
         <f aca="false">C15+$B$9*B16</f>
         <v>750</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="18" t="n">
         <f aca="false">D15+$B$9*C16</f>
         <v>1460</v>
       </c>
-      <c r="E19" s="17" t="n">
+      <c r="E19" s="18" t="n">
         <f aca="false">E15+$B$9*D16</f>
         <v>2010</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F19" s="18" t="n">
         <f aca="false">$B$9*$E$16</f>
         <v>966</v>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="G19" s="18" t="n">
         <f aca="false">$B$9*$E$16</f>
         <v>966</v>
       </c>
-      <c r="H19" s="17" t="n">
+      <c r="H19" s="18" t="n">
         <f aca="false">$B$9*$E$16</f>
         <v>966</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">B19*$B$5</f>
@@ -2265,7 +2389,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B20*$B$7</f>
@@ -2298,7 +2422,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B22" s="6" t="n">
         <f aca="false">B20*$B$8</f>
@@ -2331,75 +2455,75 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!B29</f>
+        <v>76</v>
+      </c>
+      <c r="B23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!B31</f>
         <v>27667</v>
       </c>
-      <c r="C23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!C29</f>
+      <c r="C23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!C31</f>
         <v>28184</v>
       </c>
-      <c r="D23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!D29</f>
+      <c r="D23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!D31</f>
         <v>39684</v>
       </c>
-      <c r="E23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!E29</f>
+      <c r="E23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!E31</f>
         <v>44284</v>
       </c>
-      <c r="F23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!F29</f>
+      <c r="F23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!F31</f>
         <v>9314</v>
       </c>
-      <c r="G23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!G29</f>
+      <c r="G23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!G31</f>
         <v>9314</v>
       </c>
-      <c r="H23" s="16" t="n">
-        <f aca="false">'Cost Forecast'!H29</f>
+      <c r="H23" s="17" t="n">
+        <f aca="false">'Cost Forecast'!H31</f>
         <v>14714</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" s="20" t="n">
+        <v>77</v>
+      </c>
+      <c r="B24" s="21" t="n">
         <f aca="false">B22-B23</f>
         <v>-27667</v>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="21" t="n">
         <f aca="false">C22-C23</f>
         <v>-16596.5</v>
       </c>
-      <c r="D24" s="20" t="n">
+      <c r="D24" s="21" t="n">
         <f aca="false">D22-D23</f>
         <v>-17127</v>
       </c>
-      <c r="E24" s="20" t="n">
+      <c r="E24" s="21" t="n">
         <f aca="false">E22-E23</f>
         <v>-13229.5</v>
       </c>
-      <c r="F24" s="20" t="n">
+      <c r="F24" s="21" t="n">
         <f aca="false">F22-F23</f>
         <v>5610.7</v>
       </c>
-      <c r="G24" s="20" t="n">
+      <c r="G24" s="21" t="n">
         <f aca="false">G22-G23</f>
         <v>5610.7</v>
       </c>
-      <c r="H24" s="20" t="n">
+      <c r="H24" s="21" t="n">
         <f aca="false">H22-H23</f>
         <v>210.700000000003</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25" s="21" t="n">
+        <v>78</v>
+      </c>
+      <c r="B25" s="22" t="n">
         <f aca="false">B24</f>
         <v>-27667</v>
       </c>
@@ -2423,58 +2547,58 @@
         <f aca="false">F25+G24</f>
         <v>-63398.6</v>
       </c>
-      <c r="H25" s="22" t="s">
-        <v>77</v>
+      <c r="H25" s="23" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
+      <c r="A27" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B28" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="B28" s="18" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="18" t="n">
         <f aca="false">C15+$B$10*B16</f>
         <v>750</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <f aca="false">D15+$B$10*C16</f>
         <v>1542.5</v>
       </c>
-      <c r="E28" s="17" t="n">
+      <c r="E28" s="18" t="n">
         <f aca="false">E15+$B$10*D16</f>
         <v>2230</v>
       </c>
-      <c r="F28" s="17" t="n">
+      <c r="F28" s="18" t="n">
         <f aca="false">$B$10*$E$16</f>
         <v>1345.5</v>
       </c>
-      <c r="G28" s="17" t="n">
+      <c r="G28" s="18" t="n">
         <f aca="false">$B$10*$E$16</f>
         <v>1345.5</v>
       </c>
-      <c r="H28" s="17" t="n">
+      <c r="H28" s="18" t="n">
         <f aca="false">$B$10*$E$16</f>
         <v>1345.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">B28*$B$5</f>
@@ -2507,7 +2631,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B30" s="6" t="n">
         <f aca="false">B29*$B$7</f>
@@ -2540,7 +2664,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B31" s="6" t="n">
         <f aca="false">B29*$B$8</f>
@@ -2573,75 +2697,75 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!B29</f>
+        <v>76</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!B31</f>
         <v>27667</v>
       </c>
-      <c r="C32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!C29</f>
+      <c r="C32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!C31</f>
         <v>28184</v>
       </c>
-      <c r="D32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!D29</f>
+      <c r="D32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!D31</f>
         <v>39684</v>
       </c>
-      <c r="E32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!E29</f>
+      <c r="E32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!E31</f>
         <v>44284</v>
       </c>
-      <c r="F32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!F29</f>
+      <c r="F32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!F31</f>
         <v>9314</v>
       </c>
-      <c r="G32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!G29</f>
+      <c r="G32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!G31</f>
         <v>9314</v>
       </c>
-      <c r="H32" s="16" t="n">
-        <f aca="false">'Cost Forecast'!H29</f>
+      <c r="H32" s="17" t="n">
+        <f aca="false">'Cost Forecast'!H31</f>
         <v>14714</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B33" s="20" t="n">
+        <v>77</v>
+      </c>
+      <c r="B33" s="21" t="n">
         <f aca="false">B31-B32</f>
         <v>-27667</v>
       </c>
-      <c r="C33" s="20" t="n">
+      <c r="C33" s="21" t="n">
         <f aca="false">C31-C32</f>
         <v>-16596.5</v>
       </c>
-      <c r="D33" s="20" t="n">
+      <c r="D33" s="21" t="n">
         <f aca="false">D31-D32</f>
         <v>-15852.375</v>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E33" s="21" t="n">
         <f aca="false">E31-E32</f>
         <v>-9830.5</v>
       </c>
-      <c r="F33" s="20" t="n">
+      <c r="F33" s="21" t="n">
         <f aca="false">F31-F32</f>
         <v>11473.975</v>
       </c>
-      <c r="G33" s="20" t="n">
+      <c r="G33" s="21" t="n">
         <f aca="false">G31-G32</f>
         <v>11473.975</v>
       </c>
-      <c r="H33" s="20" t="n">
+      <c r="H33" s="21" t="n">
         <f aca="false">H31-H32</f>
         <v>6073.975</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34" s="21" t="n">
+        <v>78</v>
+      </c>
+      <c r="B34" s="22" t="n">
         <f aca="false">B33</f>
         <v>-27667</v>
       </c>
@@ -2665,40 +2789,40 @@
         <f aca="false">F34+G33</f>
         <v>-46998.425</v>
       </c>
-      <c r="H34" s="22" t="s">
-        <v>77</v>
+      <c r="H34" s="23" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B38" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="C38" s="23" t="s">
+      <c r="A38" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="D38" s="23" t="s">
+      <c r="B38" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="C38" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="D38" s="24" t="s">
         <v>85</v>
       </c>
+      <c r="E38" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="F38" s="24" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="n">
+      <c r="A39" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="B39" s="17" t="n">
+      <c r="B39" s="18" t="n">
         <f aca="false">A39*$E$16</f>
         <v>517.5</v>
       </c>
@@ -2715,14 +2839,14 @@
         <v>-6718.625</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="n">
+      <c r="A40" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="B40" s="17" t="n">
+      <c r="B40" s="18" t="n">
         <f aca="false">A40*$E$16</f>
         <v>862.5</v>
       </c>
@@ -2739,14 +2863,14 @@
         <v>-1388.375</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="n">
+      <c r="A41" s="16" t="n">
         <v>0.28</v>
       </c>
-      <c r="B41" s="17" t="n">
+      <c r="B41" s="18" t="n">
         <f aca="false">A41*$E$16</f>
         <v>966</v>
       </c>
@@ -2763,14 +2887,14 @@
         <v>210.700000000003</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="n">
+      <c r="A42" s="16" t="n">
         <v>0.39</v>
       </c>
-      <c r="B42" s="17" t="n">
+      <c r="B42" s="18" t="n">
         <f aca="false">A42*$E$16</f>
         <v>1345.5</v>
       </c>
@@ -2787,12 +2911,12 @@
         <v>6073.975</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B45" s="6" t="n">
         <f aca="false">B11/B8</f>

</xml_diff>

<commit_message>
Workbook: make profit explicit on Revenue Targets sheet
- New PROFIT AT A GLANCE block: per scenario -- pilot M1-M4 investment,
  M5-M6 /mo, M7+ /mo, cumulative at M6 (NEED: -$74.6K / +$5.6K / ~$0 /
  -$63.4K; OPTIMIZE: -$69.9K / +$11.5K / +$6.1K / -$47.0K)
- Result rows renamed to MONTHLY PROFIT / LOSS and CUMULATIVE PROFIT / LOSS
- Sign-based coloring everywhere profit appears: green fill positive,
  red fill negative (Excel Good/Bad styles, conditional formatting),
  +$ prefix on positive values

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
+++ b/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="102">
   <si>
     <t xml:space="preserve">GoLuna — Path C (Anzil) Month-by-Month Cost Forecast (USD)</t>
   </si>
@@ -209,6 +209,33 @@
     <t xml:space="preserve">M7+ fixed run-rate (from Cost Forecast)</t>
   </si>
   <si>
+    <t xml:space="preserve">PROFIT — AT A GLANCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilot M1–M4 (the investment)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M5–M6 / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M7+ / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative at M6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEED — break-even (~28% ret.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPTIMIZE — compounding (~39% ret.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read: the pilot is an investment (red) in both scenarios. At the NEED line the machine reaches break-even from M7 (profit ≈ $0/mo — that is the definition of the line). At the OPTIMIZE line the same spend returns ~+$6K/mo from M7 to reinvest. Green = profit, red = loss.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metric</t>
   </si>
   <si>
@@ -254,10 +281,10 @@
     <t xml:space="preserve">Monthly cost (from Cost Forecast)</t>
   </si>
   <si>
-    <t xml:space="preserve">Operating result (net contribution − cost)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumulative result (M1–M6)</t>
+    <t xml:space="preserve">MONTHLY PROFIT / LOSS  (net contribution − cost)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUMULATIVE PROFIT / LOSS  (M1–M6)</t>
   </si>
   <si>
     <t xml:space="preserve">n/a</t>
@@ -306,12 +333,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;[RED]&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="#,##0;[RED]\(#,##0\);\-"/>
+    <numFmt numFmtId="168" formatCode="&quot;+$&quot;#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="169" formatCode="#,##0;[RED]\(#,##0\);\-"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -453,7 +481,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,10 +554,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -538,11 +562,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -551,6 +579,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -563,6 +595,38 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF006100"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <family val="0"/>
+        <b val="1"/>
+        <color rgb="FF9C0006"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -573,7 +637,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -599,12 +663,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -615,7 +679,7 @@
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF006100"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
@@ -2091,7 +2155,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -2185,749 +2249,878 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="B14" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="E14" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="20" t="n">
+        <f aca="false">SUM(B31:E31)</f>
+        <v>-74620</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <f aca="false">F31</f>
+        <v>5610.7</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <f aca="false">H31</f>
+        <v>210.700000000003</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <f aca="false">G32</f>
+        <v>-63398.6</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" s="20" t="n">
+        <f aca="false">SUM(B40:E40)</f>
+        <v>-69946.375</v>
+      </c>
+      <c r="C16" s="20" t="n">
+        <f aca="false">F40</f>
+        <v>11473.975</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <f aca="false">H40</f>
+        <v>6073.975</v>
+      </c>
+      <c r="E16" s="20" t="n">
+        <f aca="false">G41</f>
+        <v>-46998.425</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G20" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" s="17" t="n">
+      <c r="H20" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="17" t="n">
         <f aca="false">'Cost Forecast'!B27</f>
         <v>0</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C21" s="17" t="n">
         <f aca="false">'Cost Forecast'!C27</f>
         <v>15000</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D21" s="17" t="n">
         <f aca="false">'Cost Forecast'!D27</f>
         <v>25000</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E21" s="17" t="n">
         <f aca="false">'Cost Forecast'!E27</f>
         <v>29000</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F21" s="17" t="n">
         <f aca="false">'Cost Forecast'!F27</f>
         <v>0</v>
       </c>
-      <c r="G14" s="17" t="n">
+      <c r="G21" s="17" t="n">
         <f aca="false">'Cost Forecast'!G27</f>
         <v>0</v>
       </c>
-      <c r="H14" s="17" t="n">
+      <c r="H21" s="17" t="n">
         <f aca="false">'Cost Forecast'!H27</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B15" s="18" t="n">
-        <f aca="false">B14/$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <f aca="false">C14/$B$6</f>
-        <v>750</v>
-      </c>
-      <c r="D15" s="18" t="n">
-        <f aca="false">D14/$B$6</f>
-        <v>1250</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <f aca="false">E14/$B$6</f>
-        <v>1450</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <f aca="false">F14/$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="18" t="n">
-        <f aca="false">G14/$B$6</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="18" t="n">
-        <f aca="false">H14/$B$6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B16" s="18" t="n">
-        <f aca="false">B15</f>
-        <v>0</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <f aca="false">B16+C15</f>
-        <v>750</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <f aca="false">C16+D15</f>
-        <v>2000</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <f aca="false">D16+E15</f>
-        <v>3450</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <f aca="false">E16+F15</f>
-        <v>3450</v>
-      </c>
-      <c r="G16" s="18" t="n">
-        <f aca="false">F16+G15</f>
-        <v>3450</v>
-      </c>
-      <c r="H16" s="18" t="n">
-        <f aca="false">G16+H15</f>
-        <v>3450</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B19" s="18" t="n">
-        <f aca="false">0</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="18" t="n">
-        <f aca="false">C15+$B$9*B16</f>
-        <v>750</v>
-      </c>
-      <c r="D19" s="18" t="n">
-        <f aca="false">D15+$B$9*C16</f>
-        <v>1460</v>
-      </c>
-      <c r="E19" s="18" t="n">
-        <f aca="false">E15+$B$9*D16</f>
-        <v>2010</v>
-      </c>
-      <c r="F19" s="18" t="n">
-        <f aca="false">$B$9*$E$16</f>
-        <v>966</v>
-      </c>
-      <c r="G19" s="18" t="n">
-        <f aca="false">$B$9*$E$16</f>
-        <v>966</v>
-      </c>
-      <c r="H19" s="18" t="n">
-        <f aca="false">$B$9*$E$16</f>
-        <v>966</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="6" t="n">
-        <f aca="false">B19*$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <f aca="false">C19*$B$5</f>
-        <v>22500</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <f aca="false">D19*$B$5</f>
-        <v>43800</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <f aca="false">E19*$B$5</f>
-        <v>60300</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <f aca="false">F19*$B$5</f>
-        <v>28980</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <f aca="false">G19*$B$5</f>
-        <v>28980</v>
-      </c>
-      <c r="H20" s="6" t="n">
-        <f aca="false">H19*$B$5</f>
-        <v>28980</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B21" s="6" t="n">
-        <f aca="false">B20*$B$7</f>
-        <v>0</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <f aca="false">C20*$B$7</f>
-        <v>16875</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <f aca="false">D20*$B$7</f>
-        <v>32850</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <f aca="false">E20*$B$7</f>
-        <v>45225</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <f aca="false">F20*$B$7</f>
-        <v>21735</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <f aca="false">G20*$B$7</f>
-        <v>21735</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <f aca="false">H20*$B$7</f>
-        <v>21735</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="6" t="n">
-        <f aca="false">B20*$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <f aca="false">C20*$B$8</f>
-        <v>11587.5</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <f aca="false">D20*$B$8</f>
-        <v>22557</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <f aca="false">E20*$B$8</f>
-        <v>31054.5</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <f aca="false">F20*$B$8</f>
-        <v>14924.7</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <f aca="false">G20*$B$8</f>
-        <v>14924.7</v>
-      </c>
-      <c r="H22" s="6" t="n">
-        <f aca="false">H20*$B$8</f>
-        <v>14924.7</v>
+        <v>78</v>
+      </c>
+      <c r="B22" s="21" t="n">
+        <f aca="false">B21/$B$6</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="21" t="n">
+        <f aca="false">C21/$B$6</f>
+        <v>750</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <f aca="false">D21/$B$6</f>
+        <v>1250</v>
+      </c>
+      <c r="E22" s="21" t="n">
+        <f aca="false">E21/$B$6</f>
+        <v>1450</v>
+      </c>
+      <c r="F22" s="21" t="n">
+        <f aca="false">F21/$B$6</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="21" t="n">
+        <f aca="false">G21/$B$6</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="21" t="n">
+        <f aca="false">H21/$B$6</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" s="17" t="n">
+        <v>79</v>
+      </c>
+      <c r="B23" s="21" t="n">
+        <f aca="false">B22</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="21" t="n">
+        <f aca="false">B23+C22</f>
+        <v>750</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <f aca="false">C23+D22</f>
+        <v>2000</v>
+      </c>
+      <c r="E23" s="21" t="n">
+        <f aca="false">D23+E22</f>
+        <v>3450</v>
+      </c>
+      <c r="F23" s="21" t="n">
+        <f aca="false">E23+F22</f>
+        <v>3450</v>
+      </c>
+      <c r="G23" s="21" t="n">
+        <f aca="false">F23+G22</f>
+        <v>3450</v>
+      </c>
+      <c r="H23" s="21" t="n">
+        <f aca="false">G23+H22</f>
+        <v>3450</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="21" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="21" t="n">
+        <f aca="false">C22+$B$9*B23</f>
+        <v>750</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <f aca="false">D22+$B$9*C23</f>
+        <v>1460</v>
+      </c>
+      <c r="E26" s="21" t="n">
+        <f aca="false">E22+$B$9*D23</f>
+        <v>2010</v>
+      </c>
+      <c r="F26" s="21" t="n">
+        <f aca="false">$B$9*$E$23</f>
+        <v>966</v>
+      </c>
+      <c r="G26" s="21" t="n">
+        <f aca="false">$B$9*$E$23</f>
+        <v>966</v>
+      </c>
+      <c r="H26" s="21" t="n">
+        <f aca="false">$B$9*$E$23</f>
+        <v>966</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <f aca="false">B26*$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <f aca="false">C26*$B$5</f>
+        <v>22500</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <f aca="false">D26*$B$5</f>
+        <v>43800</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <f aca="false">E26*$B$5</f>
+        <v>60300</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <f aca="false">F26*$B$5</f>
+        <v>28980</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <f aca="false">G26*$B$5</f>
+        <v>28980</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <f aca="false">H26*$B$5</f>
+        <v>28980</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">B27*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <f aca="false">C27*$B$7</f>
+        <v>16875</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <f aca="false">D27*$B$7</f>
+        <v>32850</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <f aca="false">E27*$B$7</f>
+        <v>45225</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">F27*$B$7</f>
+        <v>21735</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <f aca="false">G27*$B$7</f>
+        <v>21735</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <f aca="false">H27*$B$7</f>
+        <v>21735</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <f aca="false">B27*$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <f aca="false">C27*$B$8</f>
+        <v>11587.5</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <f aca="false">D27*$B$8</f>
+        <v>22557</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <f aca="false">E27*$B$8</f>
+        <v>31054.5</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <f aca="false">F27*$B$8</f>
+        <v>14924.7</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <f aca="false">G27*$B$8</f>
+        <v>14924.7</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <f aca="false">H27*$B$8</f>
+        <v>14924.7</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="17" t="n">
         <f aca="false">'Cost Forecast'!B31</f>
         <v>27667</v>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C30" s="17" t="n">
         <f aca="false">'Cost Forecast'!C31</f>
         <v>28184</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D30" s="17" t="n">
         <f aca="false">'Cost Forecast'!D31</f>
         <v>39684</v>
       </c>
-      <c r="E23" s="17" t="n">
+      <c r="E30" s="17" t="n">
         <f aca="false">'Cost Forecast'!E31</f>
         <v>44284</v>
       </c>
-      <c r="F23" s="17" t="n">
+      <c r="F30" s="17" t="n">
         <f aca="false">'Cost Forecast'!F31</f>
         <v>9314</v>
       </c>
-      <c r="G23" s="17" t="n">
+      <c r="G30" s="17" t="n">
         <f aca="false">'Cost Forecast'!G31</f>
         <v>9314</v>
       </c>
-      <c r="H23" s="17" t="n">
+      <c r="H30" s="17" t="n">
         <f aca="false">'Cost Forecast'!H31</f>
         <v>14714</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="21" t="n">
-        <f aca="false">B22-B23</f>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="20" t="n">
+        <f aca="false">B29-B30</f>
         <v>-27667</v>
       </c>
-      <c r="C24" s="21" t="n">
-        <f aca="false">C22-C23</f>
+      <c r="C31" s="20" t="n">
+        <f aca="false">C29-C30</f>
         <v>-16596.5</v>
       </c>
-      <c r="D24" s="21" t="n">
-        <f aca="false">D22-D23</f>
+      <c r="D31" s="20" t="n">
+        <f aca="false">D29-D30</f>
         <v>-17127</v>
       </c>
-      <c r="E24" s="21" t="n">
-        <f aca="false">E22-E23</f>
+      <c r="E31" s="20" t="n">
+        <f aca="false">E29-E30</f>
         <v>-13229.5</v>
       </c>
-      <c r="F24" s="21" t="n">
-        <f aca="false">F22-F23</f>
+      <c r="F31" s="20" t="n">
+        <f aca="false">F29-F30</f>
         <v>5610.7</v>
       </c>
-      <c r="G24" s="21" t="n">
-        <f aca="false">G22-G23</f>
+      <c r="G31" s="20" t="n">
+        <f aca="false">G29-G30</f>
         <v>5610.7</v>
       </c>
-      <c r="H24" s="21" t="n">
-        <f aca="false">H22-H23</f>
+      <c r="H31" s="20" t="n">
+        <f aca="false">H29-H30</f>
         <v>210.700000000003</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25" s="22" t="n">
-        <f aca="false">B24</f>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="22" t="n">
+        <f aca="false">B31</f>
         <v>-27667</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <f aca="false">B25+C24</f>
+      <c r="C32" s="20" t="n">
+        <f aca="false">B32+C31</f>
         <v>-44263.5</v>
       </c>
-      <c r="D25" s="6" t="n">
-        <f aca="false">C25+D24</f>
+      <c r="D32" s="20" t="n">
+        <f aca="false">C32+D31</f>
         <v>-61390.5</v>
       </c>
-      <c r="E25" s="6" t="n">
-        <f aca="false">D25+E24</f>
+      <c r="E32" s="20" t="n">
+        <f aca="false">D32+E31</f>
         <v>-74620</v>
       </c>
-      <c r="F25" s="6" t="n">
-        <f aca="false">E25+F24</f>
+      <c r="F32" s="20" t="n">
+        <f aca="false">E32+F31</f>
         <v>-69009.3</v>
       </c>
-      <c r="G25" s="6" t="n">
-        <f aca="false">F25+G24</f>
+      <c r="G32" s="20" t="n">
+        <f aca="false">F32+G31</f>
         <v>-63398.6</v>
       </c>
-      <c r="H25" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B28" s="18" t="n">
+      <c r="H32" s="23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="19"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="21" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="C28" s="18" t="n">
-        <f aca="false">C15+$B$10*B16</f>
+      <c r="C35" s="21" t="n">
+        <f aca="false">C22+$B$10*B23</f>
         <v>750</v>
       </c>
-      <c r="D28" s="18" t="n">
-        <f aca="false">D15+$B$10*C16</f>
+      <c r="D35" s="21" t="n">
+        <f aca="false">D22+$B$10*C23</f>
         <v>1542.5</v>
       </c>
-      <c r="E28" s="18" t="n">
-        <f aca="false">E15+$B$10*D16</f>
+      <c r="E35" s="21" t="n">
+        <f aca="false">E22+$B$10*D23</f>
         <v>2230</v>
       </c>
-      <c r="F28" s="18" t="n">
-        <f aca="false">$B$10*$E$16</f>
+      <c r="F35" s="21" t="n">
+        <f aca="false">$B$10*$E$23</f>
         <v>1345.5</v>
       </c>
-      <c r="G28" s="18" t="n">
-        <f aca="false">$B$10*$E$16</f>
+      <c r="G35" s="21" t="n">
+        <f aca="false">$B$10*$E$23</f>
         <v>1345.5</v>
       </c>
-      <c r="H28" s="18" t="n">
-        <f aca="false">$B$10*$E$16</f>
+      <c r="H35" s="21" t="n">
+        <f aca="false">$B$10*$E$23</f>
         <v>1345.5</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B29" s="6" t="n">
-        <f aca="false">B28*$B$5</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="6" t="n">
-        <f aca="false">C28*$B$5</f>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" s="6" t="n">
+        <f aca="false">B35*$B$5</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <f aca="false">C35*$B$5</f>
         <v>22500</v>
       </c>
-      <c r="D29" s="6" t="n">
-        <f aca="false">D28*$B$5</f>
+      <c r="D36" s="6" t="n">
+        <f aca="false">D35*$B$5</f>
         <v>46275</v>
       </c>
-      <c r="E29" s="6" t="n">
-        <f aca="false">E28*$B$5</f>
+      <c r="E36" s="6" t="n">
+        <f aca="false">E35*$B$5</f>
         <v>66900</v>
       </c>
-      <c r="F29" s="6" t="n">
-        <f aca="false">F28*$B$5</f>
+      <c r="F36" s="6" t="n">
+        <f aca="false">F35*$B$5</f>
         <v>40365</v>
       </c>
-      <c r="G29" s="6" t="n">
-        <f aca="false">G28*$B$5</f>
+      <c r="G36" s="6" t="n">
+        <f aca="false">G35*$B$5</f>
         <v>40365</v>
       </c>
-      <c r="H29" s="6" t="n">
-        <f aca="false">H28*$B$5</f>
+      <c r="H36" s="6" t="n">
+        <f aca="false">H35*$B$5</f>
         <v>40365</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="B30" s="6" t="n">
-        <f aca="false">B29*$B$7</f>
-        <v>0</v>
-      </c>
-      <c r="C30" s="6" t="n">
-        <f aca="false">C29*$B$7</f>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="6" t="n">
+        <f aca="false">B36*$B$7</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <f aca="false">C36*$B$7</f>
         <v>16875</v>
       </c>
-      <c r="D30" s="6" t="n">
-        <f aca="false">D29*$B$7</f>
+      <c r="D37" s="6" t="n">
+        <f aca="false">D36*$B$7</f>
         <v>34706.25</v>
       </c>
-      <c r="E30" s="6" t="n">
-        <f aca="false">E29*$B$7</f>
+      <c r="E37" s="6" t="n">
+        <f aca="false">E36*$B$7</f>
         <v>50175</v>
       </c>
-      <c r="F30" s="6" t="n">
-        <f aca="false">F29*$B$7</f>
+      <c r="F37" s="6" t="n">
+        <f aca="false">F36*$B$7</f>
         <v>30273.75</v>
       </c>
-      <c r="G30" s="6" t="n">
-        <f aca="false">G29*$B$7</f>
+      <c r="G37" s="6" t="n">
+        <f aca="false">G36*$B$7</f>
         <v>30273.75</v>
       </c>
-      <c r="H30" s="6" t="n">
-        <f aca="false">H29*$B$7</f>
+      <c r="H37" s="6" t="n">
+        <f aca="false">H36*$B$7</f>
         <v>30273.75</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="6" t="n">
-        <f aca="false">B29*$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="C31" s="6" t="n">
-        <f aca="false">C29*$B$8</f>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" s="6" t="n">
+        <f aca="false">B36*$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <f aca="false">C36*$B$8</f>
         <v>11587.5</v>
       </c>
-      <c r="D31" s="6" t="n">
-        <f aca="false">D29*$B$8</f>
+      <c r="D38" s="6" t="n">
+        <f aca="false">D36*$B$8</f>
         <v>23831.625</v>
       </c>
-      <c r="E31" s="6" t="n">
-        <f aca="false">E29*$B$8</f>
+      <c r="E38" s="6" t="n">
+        <f aca="false">E36*$B$8</f>
         <v>34453.5</v>
       </c>
-      <c r="F31" s="6" t="n">
-        <f aca="false">F29*$B$8</f>
+      <c r="F38" s="6" t="n">
+        <f aca="false">F36*$B$8</f>
         <v>20787.975</v>
       </c>
-      <c r="G31" s="6" t="n">
-        <f aca="false">G29*$B$8</f>
+      <c r="G38" s="6" t="n">
+        <f aca="false">G36*$B$8</f>
         <v>20787.975</v>
       </c>
-      <c r="H31" s="6" t="n">
-        <f aca="false">H29*$B$8</f>
+      <c r="H38" s="6" t="n">
+        <f aca="false">H36*$B$8</f>
         <v>20787.975</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="B32" s="17" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B39" s="17" t="n">
         <f aca="false">'Cost Forecast'!B31</f>
         <v>27667</v>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C39" s="17" t="n">
         <f aca="false">'Cost Forecast'!C31</f>
         <v>28184</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D39" s="17" t="n">
         <f aca="false">'Cost Forecast'!D31</f>
         <v>39684</v>
       </c>
-      <c r="E32" s="17" t="n">
+      <c r="E39" s="17" t="n">
         <f aca="false">'Cost Forecast'!E31</f>
         <v>44284</v>
       </c>
-      <c r="F32" s="17" t="n">
+      <c r="F39" s="17" t="n">
         <f aca="false">'Cost Forecast'!F31</f>
         <v>9314</v>
       </c>
-      <c r="G32" s="17" t="n">
+      <c r="G39" s="17" t="n">
         <f aca="false">'Cost Forecast'!G31</f>
         <v>9314</v>
       </c>
-      <c r="H32" s="17" t="n">
+      <c r="H39" s="17" t="n">
         <f aca="false">'Cost Forecast'!H31</f>
         <v>14714</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="21" t="n">
-        <f aca="false">B31-B32</f>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" s="20" t="n">
+        <f aca="false">B38-B39</f>
         <v>-27667</v>
       </c>
-      <c r="C33" s="21" t="n">
-        <f aca="false">C31-C32</f>
+      <c r="C40" s="20" t="n">
+        <f aca="false">C38-C39</f>
         <v>-16596.5</v>
       </c>
-      <c r="D33" s="21" t="n">
-        <f aca="false">D31-D32</f>
+      <c r="D40" s="20" t="n">
+        <f aca="false">D38-D39</f>
         <v>-15852.375</v>
       </c>
-      <c r="E33" s="21" t="n">
-        <f aca="false">E31-E32</f>
+      <c r="E40" s="20" t="n">
+        <f aca="false">E38-E39</f>
         <v>-9830.5</v>
       </c>
-      <c r="F33" s="21" t="n">
-        <f aca="false">F31-F32</f>
+      <c r="F40" s="20" t="n">
+        <f aca="false">F38-F39</f>
         <v>11473.975</v>
       </c>
-      <c r="G33" s="21" t="n">
-        <f aca="false">G31-G32</f>
+      <c r="G40" s="20" t="n">
+        <f aca="false">G38-G39</f>
         <v>11473.975</v>
       </c>
-      <c r="H33" s="21" t="n">
-        <f aca="false">H31-H32</f>
+      <c r="H40" s="20" t="n">
+        <f aca="false">H38-H39</f>
         <v>6073.975</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B34" s="22" t="n">
-        <f aca="false">B33</f>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="22" t="n">
+        <f aca="false">B40</f>
         <v>-27667</v>
       </c>
-      <c r="C34" s="6" t="n">
-        <f aca="false">B34+C33</f>
+      <c r="C41" s="20" t="n">
+        <f aca="false">B41+C40</f>
         <v>-44263.5</v>
       </c>
-      <c r="D34" s="6" t="n">
-        <f aca="false">C34+D33</f>
+      <c r="D41" s="20" t="n">
+        <f aca="false">C41+D40</f>
         <v>-60115.875</v>
       </c>
-      <c r="E34" s="6" t="n">
-        <f aca="false">D34+E33</f>
+      <c r="E41" s="20" t="n">
+        <f aca="false">D41+E40</f>
         <v>-69946.375</v>
       </c>
-      <c r="F34" s="6" t="n">
-        <f aca="false">E34+F33</f>
+      <c r="F41" s="20" t="n">
+        <f aca="false">E41+F40</f>
         <v>-58472.4</v>
       </c>
-      <c r="G34" s="6" t="n">
-        <f aca="false">F34+G33</f>
+      <c r="G41" s="20" t="n">
+        <f aca="false">F41+G40</f>
         <v>-46998.425</v>
       </c>
-      <c r="H34" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="B38" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="C38" s="24" t="s">
-        <v>84</v>
-      </c>
-      <c r="D38" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="E38" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="F38" s="24" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="n">
+      <c r="H41" s="23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="C45" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="D45" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="E45" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="F45" s="24" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="16" t="n">
         <v>0.15</v>
       </c>
-      <c r="B39" s="18" t="n">
-        <f aca="false">A39*$E$16</f>
+      <c r="B46" s="21" t="n">
+        <f aca="false">A46*$E$23</f>
         <v>517.5</v>
       </c>
-      <c r="C39" s="6" t="n">
-        <f aca="false">B39*$B$5</f>
+      <c r="C46" s="6" t="n">
+        <f aca="false">B46*$B$5</f>
         <v>15525</v>
       </c>
-      <c r="D39" s="6" t="n">
-        <f aca="false">C39*$B$8</f>
+      <c r="D46" s="6" t="n">
+        <f aca="false">C46*$B$8</f>
         <v>7995.375</v>
       </c>
-      <c r="E39" s="6" t="n">
-        <f aca="false">D39-$B$11</f>
+      <c r="E46" s="25" t="n">
+        <f aca="false">D46-$B$11</f>
         <v>-6718.625</v>
       </c>
-      <c r="F39" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="n">
+      <c r="F46" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="16" t="n">
         <v>0.25</v>
       </c>
-      <c r="B40" s="18" t="n">
-        <f aca="false">A40*$E$16</f>
+      <c r="B47" s="21" t="n">
+        <f aca="false">A47*$E$23</f>
         <v>862.5</v>
       </c>
-      <c r="C40" s="6" t="n">
-        <f aca="false">B40*$B$5</f>
+      <c r="C47" s="6" t="n">
+        <f aca="false">B47*$B$5</f>
         <v>25875</v>
       </c>
-      <c r="D40" s="6" t="n">
-        <f aca="false">C40*$B$8</f>
+      <c r="D47" s="6" t="n">
+        <f aca="false">C47*$B$8</f>
         <v>13325.625</v>
       </c>
-      <c r="E40" s="6" t="n">
-        <f aca="false">D40-$B$11</f>
+      <c r="E47" s="25" t="n">
+        <f aca="false">D47-$B$11</f>
         <v>-1388.375</v>
       </c>
-      <c r="F40" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="n">
+      <c r="F47" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="16" t="n">
         <v>0.28</v>
       </c>
-      <c r="B41" s="18" t="n">
-        <f aca="false">A41*$E$16</f>
+      <c r="B48" s="21" t="n">
+        <f aca="false">A48*$E$23</f>
         <v>966</v>
       </c>
-      <c r="C41" s="6" t="n">
-        <f aca="false">B41*$B$5</f>
+      <c r="C48" s="6" t="n">
+        <f aca="false">B48*$B$5</f>
         <v>28980</v>
       </c>
-      <c r="D41" s="6" t="n">
-        <f aca="false">C41*$B$8</f>
+      <c r="D48" s="6" t="n">
+        <f aca="false">C48*$B$8</f>
         <v>14924.7</v>
       </c>
-      <c r="E41" s="6" t="n">
-        <f aca="false">D41-$B$11</f>
+      <c r="E48" s="25" t="n">
+        <f aca="false">D48-$B$11</f>
         <v>210.700000000003</v>
       </c>
-      <c r="F41" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="n">
+      <c r="F48" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="16" t="n">
         <v>0.39</v>
       </c>
-      <c r="B42" s="18" t="n">
-        <f aca="false">A42*$E$16</f>
+      <c r="B49" s="21" t="n">
+        <f aca="false">A49*$E$23</f>
         <v>1345.5</v>
       </c>
-      <c r="C42" s="6" t="n">
-        <f aca="false">B42*$B$5</f>
+      <c r="C49" s="6" t="n">
+        <f aca="false">B49*$B$5</f>
         <v>40365</v>
       </c>
-      <c r="D42" s="6" t="n">
-        <f aca="false">C42*$B$8</f>
+      <c r="D49" s="6" t="n">
+        <f aca="false">C49*$B$8</f>
         <v>20787.975</v>
       </c>
-      <c r="E42" s="6" t="n">
-        <f aca="false">D42-$B$11</f>
+      <c r="E49" s="25" t="n">
+        <f aca="false">D49-$B$11</f>
         <v>6073.975</v>
       </c>
-      <c r="F42" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B45" s="6" t="n">
+      <c r="F49" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B52" s="6" t="n">
         <f aca="false">B11/B8</f>
         <v>28570.8737864078</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A18:H18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B31:H31">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:G32">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B40:H40">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B41:G41">
+    <cfRule type="cellIs" priority="8" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E16">
+    <cfRule type="cellIs" priority="10" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E46:E49">
+    <cfRule type="cellIs" priority="12" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="13" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Workbook: add P&L Cascade and Fees at Scale sheets
- P&L Cascade (Path C stack): GGR -> bonuses -> NGR -> provider/crypto/PIX/
  Cubeia -> 51.5% net contribution -> fixed lines -> NET PROFIT, every line
  tagged MOVING (% of GGR, amber) or FIXED ($/mo, cyan) with who-gets-it
  notes; run at the ~$28.5K floor (NP ~= $0, kill line proven) and $100K
  (+$36,786); floor derived by formula (fixed / NC% = $28,571)
- Fees at Scale: full fee breakdown at $100K / $1M / $10M / $100M monthly
  GGR -- moving fees scale 1:1, fixed opex dilutes; net margin 16.8% ->
  26.5% -> 28.1% -> 28.5%; rates cross-linked to the cascade sheet; opex
  stepped estimates editable per column
- 353 formulas, recalc-verified zero errors

Co-Authored-By: claude-flow <ruv@ruv.net>
</commit_message>
<xml_diff>
--- a/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
+++ b/goluna-demo/Anzil_Brazil_Pilot_Forecast.xlsx
@@ -10,6 +10,8 @@
   <sheets>
     <sheet name="Cost Forecast" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Revenue Targets" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="P&amp;L Cascade" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Fees at Scale" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="175">
   <si>
     <t xml:space="preserve">GoLuna — Path C (Anzil) Month-by-Month Cost Forecast (USD)</t>
   </si>
@@ -354,6 +356,198 @@
   </si>
   <si>
     <t xml:space="preserve">M4 gate floor (GGR/mo) = M7+ run-rate ÷ net contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full P&amp;L Cascade — From GGR to Net Profit (Path C stack)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read top to bottom: every row takes a real cost out of real GGR. MOVING fees scale with revenue (% of GGR); FIXED fees are $/month regardless of revenue. Includes the ~5% high-estimate PIX on-ramp fee and treats the Cubeia €5K/mo (M7+) as additive — deliberately more conservative than the dashboard's at-scale page. Paths A/B variant: add 9% affiliate → 47.5% net, floor ~$35K.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate / $ per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At the floor (~$28.5K GGR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At $100K GGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who gets it / note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross Gaming Revenue (GGR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stakes − player wins · change the blue cells to test any level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Player bonuses &amp; incentives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOVING — % of GGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">welcome / reload / cashback — to players</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NGR  (GGR − bonuses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">what 'real' revenue actually is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Game-provider rev share (blended)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slot / live studios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Crypto processing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">processors + on-chain fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− PIX on-ramp (HIGH estimate, unconfirmed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fiat→crypto on-ramp — verify the real fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Cubeia platform rev share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">white-label platform (contract §4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NET CONTRIBUTION  (after all moving fees)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51.5% of every GGR dollar survives the moving fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Salaries (T + O + G)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIXED — $ / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− X VIP Transfer Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">staff $952 + tool $191</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Cubeia AWS hosting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€1,700/mo, Appendix B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Cubeia platform minimum (M7+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">€5K/mo from M7 — additive in this model (open question vs 'minimum')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Subscriptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer.io 324 + Freshchat 54 + security 281 + Claude 200 + other 476</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total fixed burn  (M7+ run-rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NET PROFIT / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the floor column landing at ≈ $0 is the kill line proven line-by-line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth marketing: $0 baseline after the pilot — reinvest-all means media is funded out of the Net Profit line, never the envelope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The floor, derived: fixed burn ÷ net-contribution % =</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exit M4 below this run-rate and flat → KILL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every Fee at Scale — monthly GGR of $100K / $1M / $10M / $100M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOVING fees scale 1:1 with GGR; FIXED/stepped costs dilute — that is the operating leverage. Rates link to the P&amp;L Cascade sheet (single source of truth). GoLuna fixed opex is a staffed-for-scale estimate; $100M column extrapolated (~3% of GGR) — tune to a real hiring plan. Growth marketing 20% of GGR is a steady-state assumption (media ~17.4% + Anzil 15% mgmt ~2.6%); at $5M+/mo renegotiate or in-house the 15%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth marketing (steady-state, % of GGR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type / rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$100K / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$1M / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$10M / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$100M / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Player bonuses &amp; incentives (→ players)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Game providers, blended (→ studios)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Crypto processing (→ processors)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− PIX on-ramp, high est. (→ on-ramp partner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Cubeia platform 5% (→ Cubeia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total moving fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NET CONTRIBUTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Cubeia platform minimum, M7+ (FIXED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− GoLuna fixed opex (stepped estimate — staffed for scale)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIXED / stepped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPERATING PROFIT  (EBITDA, pre-marketing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">− Growth marketing (media + Anzil 15% mgmt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net margin (% of GGR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annualised GGR (×12)</t>
   </si>
 </sst>
 </file>
@@ -368,7 +562,7 @@
     <numFmt numFmtId="168" formatCode="&quot;+$&quot;#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="169" formatCode="#,##0;[RED]\(#,##0\);\-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,8 +635,24 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF7A4D00"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF0B5563"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -470,6 +680,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEFEFEF"/>
+        <bgColor rgb="FFEDE9FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDE9C8"/>
+        <bgColor rgb="FFEFEFEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6F0F7"/>
         <bgColor rgb="FFEDE9FE"/>
       </patternFill>
     </fill>
@@ -508,7 +730,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -613,6 +835,42 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,12 +932,12 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFEFEFEF"/>
-      <rgbColor rgb="FFEDE9FE"/>
+      <rgbColor rgb="FFFDE9C8"/>
+      <rgbColor rgb="FFD6F0F7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFEDE9FE"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -689,7 +947,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFEFEFEF"/>
       <rgbColor rgb="FFC6EFCE"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -704,11 +962,11 @@
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF0B5563"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF006100"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF7A4D00"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF1F1F3A"/>
@@ -3376,4 +3634,854 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>28500</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <f aca="false">-D$5*$C6</f>
+        <v>-7125</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <f aca="false">-E$5*$C6</f>
+        <v>-25000</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="27" t="n">
+        <f aca="false">D5+D6</f>
+        <v>21375</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <f aca="false">E5+E6</f>
+        <v>75000</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <f aca="false">-D$5*$C8</f>
+        <v>-2992.5</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <f aca="false">-E$5*$C8</f>
+        <v>-10500</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <f aca="false">-D$5*$C9</f>
+        <v>-855</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <f aca="false">-E$5*$C9</f>
+        <v>-3000</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <f aca="false">-D$5*$C10</f>
+        <v>-1425</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <f aca="false">-E$5*$C10</f>
+        <v>-5000</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <f aca="false">-D$5*$C11</f>
+        <v>-1425</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <f aca="false">-E$5*$C11</f>
+        <v>-5000</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="28" t="n">
+        <f aca="false">1-C6-C8-C9-C10-C11</f>
+        <v>0.515</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <f aca="false">D5*$C12</f>
+        <v>14677.5</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <f aca="false">E5*$C12</f>
+        <v>51500</v>
+      </c>
+      <c r="F12" s="29" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <f aca="false">-$C13</f>
+        <v>-5000</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <f aca="false">-$C13</f>
+        <v>-5000</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>1143</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <f aca="false">-$C14</f>
+        <v>-1143</v>
+      </c>
+      <c r="E14" s="27" t="n">
+        <f aca="false">-$C14</f>
+        <v>-1143</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>1836</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <f aca="false">-$C15</f>
+        <v>-1836</v>
+      </c>
+      <c r="E15" s="27" t="n">
+        <f aca="false">-$C15</f>
+        <v>-1836</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>5400</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <f aca="false">-$C16</f>
+        <v>-5400</v>
+      </c>
+      <c r="E16" s="27" t="n">
+        <f aca="false">-$C16</f>
+        <v>-5400</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>1335</v>
+      </c>
+      <c r="D17" s="27" t="n">
+        <f aca="false">-$C17</f>
+        <v>-1335</v>
+      </c>
+      <c r="E17" s="27" t="n">
+        <f aca="false">-$C17</f>
+        <v>-1335</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <f aca="false">SUM(C13:C17)</f>
+        <v>14714</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <f aca="false">SUM(D13:D17)</f>
+        <v>-14714</v>
+      </c>
+      <c r="E18" s="27" t="n">
+        <f aca="false">SUM(E13:E17)</f>
+        <v>-14714</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="31" t="n">
+        <f aca="false">D12+D18</f>
+        <v>-36.5000000000036</v>
+      </c>
+      <c r="E19" s="31" t="n">
+        <f aca="false">E12+E18</f>
+        <v>36786</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <f aca="false">C18/C12</f>
+        <v>28570.8737864078</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>152</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A21:F21"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D19:E19">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B8" s="32" t="n">
+        <f aca="false">'P&amp;L Cascade'!C6</f>
+        <v>0.25</v>
+      </c>
+      <c r="C8" s="27" t="n">
+        <f aca="false">-C$7*$B8</f>
+        <v>-25000</v>
+      </c>
+      <c r="D8" s="27" t="n">
+        <f aca="false">-D$7*$B8</f>
+        <v>-250000</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <f aca="false">-E$7*$B8</f>
+        <v>-2500000</v>
+      </c>
+      <c r="F8" s="27" t="n">
+        <f aca="false">-F$7*$B8</f>
+        <v>-25000000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="32" t="n">
+        <f aca="false">'P&amp;L Cascade'!C8</f>
+        <v>0.105</v>
+      </c>
+      <c r="C9" s="27" t="n">
+        <f aca="false">-C$7*$B9</f>
+        <v>-10500</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <f aca="false">-D$7*$B9</f>
+        <v>-105000</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <f aca="false">-E$7*$B9</f>
+        <v>-1050000</v>
+      </c>
+      <c r="F9" s="27" t="n">
+        <f aca="false">-F$7*$B9</f>
+        <v>-10500000</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="32" t="n">
+        <f aca="false">'P&amp;L Cascade'!C9</f>
+        <v>0.03</v>
+      </c>
+      <c r="C10" s="27" t="n">
+        <f aca="false">-C$7*$B10</f>
+        <v>-3000</v>
+      </c>
+      <c r="D10" s="27" t="n">
+        <f aca="false">-D$7*$B10</f>
+        <v>-30000</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <f aca="false">-E$7*$B10</f>
+        <v>-300000</v>
+      </c>
+      <c r="F10" s="27" t="n">
+        <f aca="false">-F$7*$B10</f>
+        <v>-3000000</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="32" t="n">
+        <f aca="false">'P&amp;L Cascade'!C10</f>
+        <v>0.05</v>
+      </c>
+      <c r="C11" s="27" t="n">
+        <f aca="false">-C$7*$B11</f>
+        <v>-5000</v>
+      </c>
+      <c r="D11" s="27" t="n">
+        <f aca="false">-D$7*$B11</f>
+        <v>-50000</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <f aca="false">-E$7*$B11</f>
+        <v>-500000</v>
+      </c>
+      <c r="F11" s="27" t="n">
+        <f aca="false">-F$7*$B11</f>
+        <v>-5000000</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="32" t="n">
+        <f aca="false">'P&amp;L Cascade'!C11</f>
+        <v>0.05</v>
+      </c>
+      <c r="C12" s="27" t="n">
+        <f aca="false">-C$7*$B12</f>
+        <v>-5000</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <f aca="false">-D$7*$B12</f>
+        <v>-50000</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <f aca="false">-E$7*$B12</f>
+        <v>-500000</v>
+      </c>
+      <c r="F12" s="27" t="n">
+        <f aca="false">-F$7*$B12</f>
+        <v>-5000000</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="33" t="n">
+        <f aca="false">SUM(B8:B12)</f>
+        <v>0.485</v>
+      </c>
+      <c r="C13" s="27" t="n">
+        <f aca="false">SUM(C8:C12)</f>
+        <v>-48500</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <f aca="false">SUM(D8:D12)</f>
+        <v>-485000</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <f aca="false">SUM(E8:E12)</f>
+        <v>-4850000</v>
+      </c>
+      <c r="F13" s="27" t="n">
+        <f aca="false">SUM(F8:F12)</f>
+        <v>-48500000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="28" t="n">
+        <f aca="false">1-B13</f>
+        <v>0.515</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <f aca="false">C7+C13</f>
+        <v>51500</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">D7+D13</f>
+        <v>515000</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <f aca="false">E7+E13</f>
+        <v>5150000</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <f aca="false">F7+F13</f>
+        <v>51500000</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <f aca="false">'P&amp;L Cascade'!C16</f>
+        <v>5400</v>
+      </c>
+      <c r="C15" s="27" t="n">
+        <f aca="false">-$B15</f>
+        <v>-5400</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <f aca="false">-$B15</f>
+        <v>-5400</v>
+      </c>
+      <c r="E15" s="27" t="n">
+        <f aca="false">-$B15</f>
+        <v>-5400</v>
+      </c>
+      <c r="F15" s="27" t="n">
+        <f aca="false">-$B15</f>
+        <v>-5400</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-9314</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>-45000</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>-330000</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>-3000000</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <f aca="false">C14+C15+C16</f>
+        <v>36786</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <f aca="false">D14+D15+D16</f>
+        <v>464600</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <f aca="false">E14+E15+E16</f>
+        <v>4814600</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <f aca="false">F14+F15+F16</f>
+        <v>48494600</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B18" s="33" t="n">
+        <f aca="false">B4</f>
+        <v>0.2</v>
+      </c>
+      <c r="C18" s="27" t="n">
+        <f aca="false">-C$7*$B$4</f>
+        <v>-20000</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <f aca="false">-D$7*$B$4</f>
+        <v>-200000</v>
+      </c>
+      <c r="E18" s="27" t="n">
+        <f aca="false">-E$7*$B$4</f>
+        <v>-2000000</v>
+      </c>
+      <c r="F18" s="27" t="n">
+        <f aca="false">-F$7*$B$4</f>
+        <v>-20000000</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="31" t="n">
+        <f aca="false">C17+C18</f>
+        <v>16786</v>
+      </c>
+      <c r="D19" s="31" t="n">
+        <f aca="false">D17+D18</f>
+        <v>264600</v>
+      </c>
+      <c r="E19" s="31" t="n">
+        <f aca="false">E17+E18</f>
+        <v>2814600</v>
+      </c>
+      <c r="F19" s="31" t="n">
+        <f aca="false">F17+F18</f>
+        <v>28494600</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C20" s="33" t="n">
+        <f aca="false">C19/C7</f>
+        <v>0.16786</v>
+      </c>
+      <c r="D20" s="33" t="n">
+        <f aca="false">D19/D7</f>
+        <v>0.2646</v>
+      </c>
+      <c r="E20" s="33" t="n">
+        <f aca="false">E19/E7</f>
+        <v>0.28146</v>
+      </c>
+      <c r="F20" s="33" t="n">
+        <f aca="false">F19/F7</f>
+        <v>0.284946</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" s="34" t="n">
+        <f aca="false">C7*12</f>
+        <v>1200000</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <f aca="false">D7*12</f>
+        <v>12000000</v>
+      </c>
+      <c r="E21" s="34" t="n">
+        <f aca="false">E7*12</f>
+        <v>120000000</v>
+      </c>
+      <c r="F21" s="34" t="n">
+        <f aca="false">F7*12</f>
+        <v>1200000000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C17:F17">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:F19">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>